<commit_message>
regdb: Update to Pong_B4.1-260414-1749
Signed-off-by: Omkar Chandorkar <gotenksIN@aospa.co>
</commit_message>
<xml_diff>
--- a/wlan/phyrf_svc/tools/bdfUtil/Regulatory_BDF_tools/Regulatory_BDF_6G_In_Data.xlsx
+++ b/wlan/phyrf_svc/tools/bdfUtil/Regulatory_BDF_tools/Regulatory_BDF_6G_In_Data.xlsx
@@ -1,36 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="30720" yWindow="1920" windowWidth="21600" windowHeight="11235" tabRatio="770" firstSheet="6" activeTab="7" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="REGDB_VERSION_HISTORY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="REG_DOMAINS_2G_LOOKUP" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="REG_DOMAINS_5G_LOOKUP" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="REG_DOMAINS_6G_LOOKUP" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="REG_DOMAIN_PAIRS_INPUT" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SUPER_DOMAIN_INPUT" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="REG_RULES_2G_LOOKUP" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="REG_RULES_5G_LOOKUP" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="REG_RULES_6G_LOOKUP" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="IMPORTANT_MACROS_LOOKUP" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="DFS_LOOKUP" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="CTL_LOOKUP" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="COUNTRY_LOOKUP" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="REG_DMN_PAIR_LOOKUP" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="SUPER_DMN_6G_LOOKUP" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="ALL_COUNTRIES_INPUT" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="REG_RULES_2G_INPUT" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="REG_DOMAINS_2G_INPUT" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="REG_RULES_5G_INPUT" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="REG_DOMAINS_5G_INPUT" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="REG_DOMAINS_6G_INPUT" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="REG_RULES_6G_INPUT" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="SUBDOMAINS_6G_MAP" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="SUBDOMAINS_6G_INPUT" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="5G6GBWCONVERTER" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REGDB_VERSION_HISTORY" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_DOMAINS_2G_LOOKUP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_DOMAINS_5G_LOOKUP" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_DOMAINS_6G_LOOKUP" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_DOMAIN_PAIRS_INPUT" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUPER_DOMAIN_INPUT" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_RULES_2G_LOOKUP" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_RULES_5G_LOOKUP" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_RULES_6G_LOOKUP" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IMPORTANT_MACROS_LOOKUP" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DFS_LOOKUP" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CTL_LOOKUP" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COUNTRY_LOOKUP" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_DMN_PAIR_LOOKUP" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUPER_DMN_6G_LOOKUP" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALL_COUNTRIES_INPUT" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_RULES_2G_INPUT" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_DOMAINS_2G_INPUT" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_RULES_5G_INPUT" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_DOMAINS_5G_INPUT" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_DOMAINS_6G_INPUT" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REG_RULES_6G_INPUT" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUBDOMAINS_6G_MAP" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUBDOMAINS_6G_INPUT" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5G6GBWCONVERTER" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'REG_RULES_5G_INPUT'!$A$1:$H$141</definedName>
@@ -22955,6 +22955,9 @@
       <c r="F49" t="n">
         <v>0</v>
       </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>CHAN_5170_5250_2</t>

</xml_diff>

<commit_message>
Import lost changes from WLAN.HSP.2.0.c10-00465-QCAHSPSWPL_V1_V2_SILICONZ-1 after switching to Pong
Signed-off-by: Omkar Chandorkar <gotenksIN@aospa.co>
</commit_message>
<xml_diff>
--- a/wlan/phyrf_svc/tools/bdfUtil/Regulatory_BDF_tools/Regulatory_BDF_6G_In_Data.xlsx
+++ b/wlan/phyrf_svc/tools/bdfUtil/Regulatory_BDF_tools/Regulatory_BDF_6G_In_Data.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="C1" s="6" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D1" t="inlineStr">
         <is>
@@ -8030,7 +8030,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -8050,7 +8050,7 @@
         <v>160</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -8092,7 +8092,7 @@
         <v>160</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -8240,7 +8240,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -8260,7 +8260,7 @@
         <v>160</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -8324,7 +8324,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -8344,7 +8344,7 @@
         <v>160</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -8576,7 +8576,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -8596,7 +8596,7 @@
         <v>160</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -9374,7 +9374,7 @@
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -9394,7 +9394,7 @@
         <v>160</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I42" t="n">
         <v>0</v>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -10528,7 +10528,7 @@
         <v>160</v>
       </c>
       <c r="H69" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I69" t="n">
         <v>0</v>
@@ -10592,7 +10592,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -10612,7 +10612,7 @@
         <v>160</v>
       </c>
       <c r="H71" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I71" t="n">
         <v>0</v>
@@ -10634,7 +10634,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -10654,7 +10654,7 @@
         <v>160</v>
       </c>
       <c r="H72" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I72" t="n">
         <v>0</v>
@@ -10676,7 +10676,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -10696,7 +10696,7 @@
         <v>160</v>
       </c>
       <c r="H73" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I73" t="n">
         <v>0</v>
@@ -10760,7 +10760,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -10780,7 +10780,7 @@
         <v>160</v>
       </c>
       <c r="H75" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I75" t="n">
         <v>0</v>
@@ -11012,7 +11012,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -11032,7 +11032,7 @@
         <v>160</v>
       </c>
       <c r="H81" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I81" t="n">
         <v>0</v>
@@ -11096,7 +11096,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -11116,7 +11116,7 @@
         <v>160</v>
       </c>
       <c r="H83" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I83" t="n">
         <v>0</v>
@@ -11558,7 +11558,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -11578,7 +11578,7 @@
         <v>160</v>
       </c>
       <c r="H94" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I94" t="n">
         <v>0</v>
@@ -11936,7 +11936,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11956,7 +11956,7 @@
         <v>160</v>
       </c>
       <c r="H103" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I103" t="n">
         <v>0</v>
@@ -12188,7 +12188,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -12208,7 +12208,7 @@
         <v>160</v>
       </c>
       <c r="H109" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I109" t="n">
         <v>0</v>
@@ -12692,7 +12692,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -12712,7 +12712,7 @@
         <v>160</v>
       </c>
       <c r="H121" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I121" t="n">
         <v>0</v>
@@ -12776,7 +12776,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -12796,7 +12796,7 @@
         <v>160</v>
       </c>
       <c r="H123" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I123" t="n">
         <v>0</v>
@@ -12818,7 +12818,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -12838,7 +12838,7 @@
         <v>160</v>
       </c>
       <c r="H124" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I124" t="n">
         <v>0</v>
@@ -13070,7 +13070,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -13090,7 +13090,7 @@
         <v>160</v>
       </c>
       <c r="H130" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I130" t="n">
         <v>0</v>
@@ -13910,7 +13910,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -13930,7 +13930,7 @@
         <v>160</v>
       </c>
       <c r="H150" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I150" t="n">
         <v>0</v>
@@ -14162,7 +14162,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -14182,7 +14182,7 @@
         <v>160</v>
       </c>
       <c r="H156" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I156" t="n">
         <v>0</v>
@@ -14330,7 +14330,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -14350,7 +14350,7 @@
         <v>160</v>
       </c>
       <c r="H160" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I160" t="n">
         <v>0</v>
@@ -14372,7 +14372,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -14392,7 +14392,7 @@
         <v>160</v>
       </c>
       <c r="H161" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I161" t="n">
         <v>0</v>
@@ -14582,7 +14582,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -14602,7 +14602,7 @@
         <v>160</v>
       </c>
       <c r="H166" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I166" t="n">
         <v>0</v>
@@ -14792,7 +14792,7 @@
       </c>
       <c r="C171" s="13" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -14812,7 +14812,7 @@
         <v>160</v>
       </c>
       <c r="H171" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I171" t="n">
         <v>0</v>
@@ -14876,7 +14876,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -14896,7 +14896,7 @@
         <v>160</v>
       </c>
       <c r="H173" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I173" t="n">
         <v>0</v>
@@ -14918,7 +14918,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -14938,7 +14938,7 @@
         <v>160</v>
       </c>
       <c r="H174" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I174" t="n">
         <v>0</v>
@@ -14960,7 +14960,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -14980,7 +14980,7 @@
         <v>160</v>
       </c>
       <c r="H175" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I175" t="n">
         <v>0</v>
@@ -15044,7 +15044,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -15064,7 +15064,7 @@
         <v>160</v>
       </c>
       <c r="H177" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I177" t="n">
         <v>0</v>
@@ -15086,7 +15086,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -15106,7 +15106,7 @@
         <v>160</v>
       </c>
       <c r="H178" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I178" t="n">
         <v>0</v>
@@ -15254,7 +15254,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -15274,7 +15274,7 @@
         <v>160</v>
       </c>
       <c r="H182" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I182" t="n">
         <v>0</v>
@@ -15338,7 +15338,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -15358,7 +15358,7 @@
         <v>160</v>
       </c>
       <c r="H184" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I184" t="n">
         <v>0</v>
@@ -15380,7 +15380,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -15400,7 +15400,7 @@
         <v>40</v>
       </c>
       <c r="H185" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I185" t="n">
         <v>0</v>
@@ -15506,7 +15506,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -15526,7 +15526,7 @@
         <v>160</v>
       </c>
       <c r="H188" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I188" t="n">
         <v>0</v>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -15946,7 +15946,7 @@
         <v>160</v>
       </c>
       <c r="H198" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I198" t="n">
         <v>0</v>
@@ -16388,7 +16388,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -16408,7 +16408,7 @@
         <v>160</v>
       </c>
       <c r="H209" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I209" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Enable missing channels from currently latest wireless-regdb
https://git.kernel.org/pub/scm/linux/kernel/git/wens/wireless-regdb.git/plain/db.txt?id=d0781152c3349d64faffaaa28d1221eafe389346

Signed-off-by: Omkar Chandorkar <gotenksIN@aospa.co>
</commit_message>
<xml_diff>
--- a/wlan/phyrf_svc/tools/bdfUtil/Regulatory_BDF_tools/Regulatory_BDF_6G_In_Data.xlsx
+++ b/wlan/phyrf_svc/tools/bdfUtil/Regulatory_BDF_tools/Regulatory_BDF_6G_In_Data.xlsx
@@ -7778,7 +7778,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -7798,7 +7798,7 @@
         <v>160</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -8198,7 +8198,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -8218,7 +8218,7 @@
         <v>160</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -8702,7 +8702,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -8722,7 +8722,7 @@
         <v>160</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -9626,7 +9626,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -9646,7 +9646,7 @@
         <v>160</v>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I48" t="n">
         <v>0</v>
@@ -11348,7 +11348,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>FCC_6G_1</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -11368,7 +11368,7 @@
         <v>80</v>
       </c>
       <c r="H89" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I89" t="n">
         <v>0</v>
@@ -11726,7 +11726,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -11746,7 +11746,7 @@
         <v>160</v>
       </c>
       <c r="H98" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I98" t="n">
         <v>0</v>
@@ -12230,7 +12230,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>FCC_6G_1</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -12250,7 +12250,7 @@
         <v>160</v>
       </c>
       <c r="H110" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I110" t="n">
         <v>0</v>
@@ -12272,7 +12272,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -12292,7 +12292,7 @@
         <v>160</v>
       </c>
       <c r="H111" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I111" t="n">
         <v>0</v>
@@ -12902,7 +12902,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -12922,7 +12922,7 @@
         <v>160</v>
       </c>
       <c r="H126" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I126" t="n">
         <v>0</v>
@@ -13574,7 +13574,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -13594,7 +13594,7 @@
         <v>160</v>
       </c>
       <c r="H142" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I142" t="n">
         <v>0</v>
@@ -13616,7 +13616,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>FCC_6G_1</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -13636,7 +13636,7 @@
         <v>160</v>
       </c>
       <c r="H143" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I143" t="n">
         <v>0</v>
@@ -13784,7 +13784,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>FCC_6G_1</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -13804,7 +13804,7 @@
         <v>160</v>
       </c>
       <c r="H147" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I147" t="n">
         <v>0</v>
@@ -13868,7 +13868,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>FCC_6G_1</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -13888,7 +13888,7 @@
         <v>160</v>
       </c>
       <c r="H149" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I149" t="n">
         <v>0</v>
@@ -14120,7 +14120,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -14140,7 +14140,7 @@
         <v>160</v>
       </c>
       <c r="H155" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I155" t="n">
         <v>0</v>
@@ -14750,7 +14750,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -14770,7 +14770,7 @@
         <v>160</v>
       </c>
       <c r="H170" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I170" t="n">
         <v>0</v>
@@ -15296,7 +15296,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -15316,7 +15316,7 @@
         <v>160</v>
       </c>
       <c r="H183" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I183" t="n">
         <v>0</v>
@@ -15464,7 +15464,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -15484,7 +15484,7 @@
         <v>160</v>
       </c>
       <c r="H187" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I187" t="n">
         <v>0</v>
@@ -15632,7 +15632,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>ETSI_6G_1</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -15652,7 +15652,7 @@
         <v>160</v>
       </c>
       <c r="H191" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I191" t="n">
         <v>0</v>
@@ -16010,7 +16010,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>NULL_6G</t>
+          <t>FCC_6G_1</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -16030,7 +16030,7 @@
         <v>160</v>
       </c>
       <c r="H200" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I200" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
regdb: Explicitly set FCC 6GHz LPI rule
</commit_message>
<xml_diff>
--- a/wlan/phyrf_svc/tools/bdfUtil/Regulatory_BDF_tools/Regulatory_BDF_6G_In_Data.xlsx
+++ b/wlan/phyrf_svc/tools/bdfUtil/Regulatory_BDF_tools/Regulatory_BDF_6G_In_Data.xlsx
@@ -24626,6 +24626,11 @@
       <c r="E3" t="n">
         <v>320</v>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CHAN_5925_7125_1</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">

</xml_diff>